<commit_message>
feat(SP lane 4): the kit writes the ARR to recognised revenue bridge itself
arr_to_revenue.csv for the as of month, plus a section in report.md and
closepack.md: schedule MRR, less each bucket, = supported; plus each bucket,
= invoiced recurring; = recognised from the roll forward; billings to recognised
through the deferred movement; one off lines as a memo row. Every amount is a
sum of columns already in compare_customer_month.csv and deferred_rollforward.csv;
a gap prints as a residual row.

Larkspur 2025-10: 72,400 - 2,100 - 800 = 69,500 + 1,400 + 300 + 950 = 72,150,
residual 0, as ARR-TO-GAAP-BRIDGE.md states. All four committed examples
regenerated, all four receipts verify; no existing figure moved.
example/check_arr_to_revenue.py: 64 ok; fails on a mutant that moves 100
between two steps, with or without the residual row.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/example/next_month/out/pilot.xlsx
+++ b/example/next_month/out/pilot.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions by cause" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retention" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohorts" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Match" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer month" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deferred" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deferred by account" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bridge" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Exceptions by cause" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Accounts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Retention" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Cohorts" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Match" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Customer month" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Deferred" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Deferred by account" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Bridge" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,16 +26,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,7 +43,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -54,21 +51,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,22 +426,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>reported_arr</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>supported_arr</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>unresolved_arr</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>asof</t>
         </is>
@@ -490,47 +478,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>basis</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>start</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>new</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>reactivation</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>expansion</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>contraction</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>churn</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>end</t>
         </is>
@@ -2135,17 +2123,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dominant_cause</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>accounts</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>unresolved_arr</t>
         </is>
@@ -2257,62 +2245,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>key</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>customer_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>customer_name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>asof_schedule_mrr</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>asof_invoice_mrr</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>asof_supported_mrr</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>asof_unresolved_mrr</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>months_in_window</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>months_not_supported</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>dominant_cause</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>causes</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>net_diff_window</t>
         </is>
@@ -4293,47 +4281,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>basis</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>period_from</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>period_to</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>starting_book_mrr</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>starting_accounts</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ending_mrr_same_accounts</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>churned_accounts</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>GRR</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>NRR</t>
         </is>
@@ -4459,22 +4447,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>cohort</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>accounts</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>revenue_retained_12m_schedule_pct</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>revenue_retained_12m_supported_pct</t>
         </is>
@@ -4511,32 +4499,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>sched_key</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>inv_key</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>sched_name</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>inv_name</t>
         </is>
@@ -5941,92 +5929,92 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>key</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>cid</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>cname</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>sched_mrr</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>inv_key</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>inv_recurring</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>inv_credit</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>has_credit</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>has_duplicate_id</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>has_no_period</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>inv_mrr</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>non_recurring_amount</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>unknown_lines</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>diff</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>supported_mrr</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>bucket</t>
         </is>
@@ -46601,37 +46589,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>opening</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>billings</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>recognised</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>closing</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>closing_deferred</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>closing_unbilled</t>
         </is>
@@ -46952,27 +46940,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>key</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>customer_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>closing_deferred</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>closing_unbilled</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>months_of_deferred_cover</t>
         </is>

</xml_diff>